<commit_message>
Se actualizan componentes y archivos principales
</commit_message>
<xml_diff>
--- a/src/excel/BDAdolecente.xlsx
+++ b/src/excel/BDAdolecente.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wgonzalez\Virtual_host\Sorteo\fuentes\src\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wgonzalez\Virtual_host\sorteo-ciclos-deliberativos\src\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24537EA7-8A51-405F-A2F7-0354FBB778DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AA3423F-6223-46C9-A324-24E427391DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,15 +33,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>Id</t>
   </si>
   <si>
     <t>Número de Identificación</t>
-  </si>
-  <si>
-    <t>1012394837</t>
   </si>
   <si>
     <t>1022968945</t>
@@ -218,10 +215,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -248,8 +244,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:B47" totalsRowShown="0">
-  <autoFilter ref="A1:B47" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:B46" totalsRowShown="0">
+  <autoFilter ref="A1:B46" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="1">
       <extLst>
@@ -591,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="20" bestFit="1" customWidth="1"/>
@@ -607,71 +603,71 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>12</v>
@@ -679,7 +675,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>13</v>
@@ -687,7 +683,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>14</v>
@@ -695,7 +691,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>15</v>
@@ -703,7 +699,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>16</v>
@@ -711,7 +707,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>17</v>
@@ -719,7 +715,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>18</v>
@@ -727,7 +723,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>19</v>
@@ -735,7 +731,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B18" t="s">
         <v>20</v>
@@ -743,7 +739,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>21</v>
@@ -751,39 +747,39 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>25</v>
@@ -791,103 +787,103 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>3</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>37</v>
@@ -895,7 +891,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>38</v>
@@ -903,7 +899,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>39</v>
@@ -911,7 +907,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>40</v>
@@ -919,58 +915,50 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="2">
-        <v>41</v>
-      </c>
-      <c r="B42" s="3" t="s">
+      <c r="A42">
+        <v>46</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
-        <v>42</v>
-      </c>
-      <c r="B43" s="3" t="s">
+      <c r="A43">
+        <v>47</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="2">
-        <v>43</v>
-      </c>
-      <c r="B44" s="3" t="s">
+      <c r="A44">
+        <v>48</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="2">
-        <v>44</v>
-      </c>
-      <c r="B45" s="3" t="s">
+      <c r="A45">
+        <v>50</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="2">
-        <v>45</v>
-      </c>
-      <c r="B46" s="3" t="s">
+      <c r="A46">
+        <v>51</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>46</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="2">
-        <v>46</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>